<commit_message>
Update data mikro sls
</commit_message>
<xml_diff>
--- a/research/fasih-dashboard-se2026/data_mikro_sls/Agregat_Kecamatan_ANGGOTA KELUARGA.xlsx
+++ b/research/fasih-dashboard-se2026/data_mikro_sls/Agregat_Kecamatan_ANGGOTA KELUARGA.xlsx
@@ -612,100 +612,100 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>4684</v>
+        <v>5445</v>
       </c>
       <c r="D2" t="n">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="E2" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="F2" t="n">
-        <v>135</v>
+        <v>166</v>
       </c>
       <c r="G2" t="n">
         <v>1</v>
       </c>
       <c r="H2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>4753</v>
+        <v>5532</v>
       </c>
       <c r="K2" t="n">
-        <v>1516</v>
+        <v>1281</v>
       </c>
       <c r="L2" t="n">
-        <v>1858</v>
+        <v>1819</v>
       </c>
       <c r="M2" t="n">
-        <v>351</v>
+        <v>357</v>
       </c>
       <c r="N2" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="O2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P2" t="n">
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="R2" t="n">
         <v>3</v>
       </c>
       <c r="S2" t="n">
-        <v>267</v>
+        <v>589</v>
       </c>
       <c r="T2" t="n">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="U2" t="n">
-        <v>4044</v>
+        <v>4118</v>
       </c>
       <c r="V2" t="n">
-        <v>2491</v>
+        <v>2798</v>
       </c>
       <c r="W2" t="n">
-        <v>1491</v>
+        <v>1283</v>
       </c>
       <c r="X2" t="n">
-        <v>1763</v>
+        <v>1819</v>
       </c>
       <c r="Y2" t="n">
-        <v>327</v>
+        <v>354</v>
       </c>
       <c r="Z2" t="n">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="AA2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB2" t="n">
         <v>0</v>
       </c>
       <c r="AC2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AD2" t="n">
         <v>3</v>
       </c>
       <c r="AE2" t="n">
-        <v>407</v>
+        <v>589</v>
       </c>
       <c r="AF2" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="AG2" t="n">
-        <v>4054</v>
+        <v>4118</v>
       </c>
       <c r="AH2" t="n">
-        <v>2515</v>
+        <v>2795</v>
       </c>
     </row>
     <row r="3">
@@ -720,16 +720,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>994</v>
+        <v>1108</v>
       </c>
       <c r="D3" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E3" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F3" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="G3" t="n">
         <v>1</v>
@@ -741,79 +741,79 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>1024</v>
+        <v>1139</v>
       </c>
       <c r="K3" t="n">
-        <v>464</v>
+        <v>451</v>
       </c>
       <c r="L3" t="n">
-        <v>513</v>
+        <v>433</v>
       </c>
       <c r="M3" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="N3" t="n">
-        <v>330</v>
+        <v>298</v>
       </c>
       <c r="O3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="P3" t="n">
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R3" t="n">
         <v>1</v>
       </c>
       <c r="S3" t="n">
-        <v>84</v>
+        <v>205</v>
       </c>
       <c r="T3" t="n">
         <v>0</v>
       </c>
       <c r="U3" t="n">
-        <v>1408</v>
+        <v>1410</v>
       </c>
       <c r="V3" t="n">
-        <v>614</v>
+        <v>661</v>
       </c>
       <c r="W3" t="n">
-        <v>464</v>
+        <v>442</v>
       </c>
       <c r="X3" t="n">
-        <v>514</v>
+        <v>446</v>
       </c>
       <c r="Y3" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="Z3" t="n">
-        <v>329</v>
+        <v>298</v>
       </c>
       <c r="AA3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AB3" t="n">
         <v>0</v>
       </c>
       <c r="AC3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AD3" t="n">
         <v>1</v>
       </c>
       <c r="AE3" t="n">
-        <v>83</v>
+        <v>205</v>
       </c>
       <c r="AF3" t="n">
         <v>0</v>
       </c>
       <c r="AG3" t="n">
-        <v>1408</v>
+        <v>1410</v>
       </c>
       <c r="AH3" t="n">
-        <v>615</v>
+        <v>670</v>
       </c>
     </row>
     <row r="4">
@@ -828,46 +828,46 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>5146</v>
+        <v>6119</v>
       </c>
       <c r="D4" t="n">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="E4" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="F4" t="n">
-        <v>559</v>
+        <v>677</v>
       </c>
       <c r="G4" t="n">
         <v>7</v>
       </c>
       <c r="H4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>5227</v>
+        <v>6210</v>
       </c>
       <c r="K4" t="n">
-        <v>2208</v>
+        <v>1831</v>
       </c>
       <c r="L4" t="n">
-        <v>3449</v>
+        <v>3389</v>
       </c>
       <c r="M4" t="n">
-        <v>92</v>
+        <v>359</v>
       </c>
       <c r="N4" t="n">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="O4" t="n">
-        <v>76</v>
+        <v>53</v>
       </c>
       <c r="P4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q4" t="n">
         <v>0</v>
@@ -876,34 +876,34 @@
         <v>0</v>
       </c>
       <c r="S4" t="n">
+        <v>422</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" t="n">
+        <v>6152</v>
+      </c>
+      <c r="V4" t="n">
+        <v>4225</v>
+      </c>
+      <c r="W4" t="n">
+        <v>1756</v>
+      </c>
+      <c r="X4" t="n">
+        <v>3456</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>386</v>
+      </c>
+      <c r="Z4" t="n">
         <v>95</v>
       </c>
-      <c r="T4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U4" t="n">
-        <v>6010</v>
-      </c>
-      <c r="V4" t="n">
-        <v>3715</v>
-      </c>
-      <c r="W4" t="n">
-        <v>2208</v>
-      </c>
-      <c r="X4" t="n">
-        <v>3445</v>
-      </c>
-      <c r="Y4" t="n">
-        <v>96</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>88</v>
-      </c>
       <c r="AA4" t="n">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="AB4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AC4" t="n">
         <v>0</v>
@@ -912,16 +912,16 @@
         <v>0</v>
       </c>
       <c r="AE4" t="n">
-        <v>95</v>
+        <v>422</v>
       </c>
       <c r="AF4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG4" t="n">
-        <v>6010</v>
+        <v>6181</v>
       </c>
       <c r="AH4" t="n">
-        <v>3714</v>
+        <v>4330</v>
       </c>
     </row>
     <row r="5">
@@ -936,16 +936,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>3095</v>
+        <v>3542</v>
       </c>
       <c r="D5" t="n">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="E5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F5" t="n">
-        <v>166</v>
+        <v>204</v>
       </c>
       <c r="G5" t="n">
         <v>2</v>
@@ -957,16 +957,16 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>3149</v>
+        <v>3611</v>
       </c>
       <c r="K5" t="n">
-        <v>1070</v>
+        <v>902</v>
       </c>
       <c r="L5" t="n">
-        <v>1615</v>
+        <v>1675</v>
       </c>
       <c r="M5" t="n">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="N5" t="n">
         <v>0</v>
@@ -978,31 +978,31 @@
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
       </c>
       <c r="S5" t="n">
-        <v>250</v>
+        <v>440</v>
       </c>
       <c r="T5" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="U5" t="n">
-        <v>3058</v>
+        <v>3121</v>
       </c>
       <c r="V5" t="n">
-        <v>1988</v>
+        <v>2219</v>
       </c>
       <c r="W5" t="n">
-        <v>1070</v>
+        <v>902</v>
       </c>
       <c r="X5" t="n">
-        <v>1620</v>
+        <v>1675</v>
       </c>
       <c r="Y5" t="n">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="Z5" t="n">
         <v>0</v>
@@ -1014,22 +1014,22 @@
         <v>0</v>
       </c>
       <c r="AC5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AD5" t="n">
         <v>0</v>
       </c>
       <c r="AE5" t="n">
-        <v>246</v>
+        <v>440</v>
       </c>
       <c r="AF5" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="AG5" t="n">
-        <v>3058</v>
+        <v>3121</v>
       </c>
       <c r="AH5" t="n">
-        <v>1988</v>
+        <v>2219</v>
       </c>
     </row>
     <row r="6">
@@ -1044,100 +1044,100 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>839</v>
+        <v>1114</v>
       </c>
       <c r="D6" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="E6" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F6" t="n">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="G6" t="n">
         <v>3</v>
       </c>
       <c r="H6" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>859</v>
+        <v>1138</v>
       </c>
       <c r="K6" t="n">
-        <v>542</v>
+        <v>448</v>
       </c>
       <c r="L6" t="n">
-        <v>486</v>
+        <v>544</v>
       </c>
       <c r="M6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="O6" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="P6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>1</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" t="n">
+        <v>93</v>
+      </c>
+      <c r="T6" t="n">
+        <v>8</v>
+      </c>
+      <c r="U6" t="n">
+        <v>1121</v>
+      </c>
+      <c r="V6" t="n">
+        <v>659</v>
+      </c>
+      <c r="W6" t="n">
+        <v>449</v>
+      </c>
+      <c r="X6" t="n">
+        <v>544</v>
+      </c>
+      <c r="Y6" t="n">
         <v>5</v>
       </c>
-      <c r="Q6" t="n">
-        <v>2</v>
-      </c>
-      <c r="R6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S6" t="n">
-        <v>44</v>
-      </c>
-      <c r="T6" t="n">
-        <v>6</v>
-      </c>
-      <c r="U6" t="n">
-        <v>1105</v>
-      </c>
-      <c r="V6" t="n">
-        <v>550</v>
-      </c>
-      <c r="W6" t="n">
-        <v>543</v>
-      </c>
-      <c r="X6" t="n">
-        <v>490</v>
-      </c>
-      <c r="Y6" t="n">
-        <v>6</v>
-      </c>
       <c r="Z6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AA6" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="AB6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AC6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AD6" t="n">
         <v>0</v>
       </c>
       <c r="AE6" t="n">
-        <v>40</v>
+        <v>92</v>
       </c>
       <c r="AF6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="AG6" t="n">
-        <v>1105</v>
+        <v>1121</v>
       </c>
       <c r="AH6" t="n">
-        <v>549</v>
+        <v>658</v>
       </c>
     </row>
     <row r="7">
@@ -1152,46 +1152,46 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>892</v>
+        <v>1029</v>
       </c>
       <c r="D7" t="n">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="E7" t="n">
+        <v>9</v>
+      </c>
+      <c r="F7" t="n">
+        <v>47</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
         <v>8</v>
       </c>
-      <c r="F7" t="n">
-        <v>45</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" t="n">
-        <v>5</v>
-      </c>
       <c r="I7" t="n">
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>931</v>
+        <v>1076</v>
       </c>
       <c r="K7" t="n">
-        <v>428</v>
+        <v>394</v>
       </c>
       <c r="L7" t="n">
-        <v>510</v>
+        <v>498</v>
       </c>
       <c r="M7" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="N7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>
       </c>
       <c r="P7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q7" t="n">
         <v>0</v>
@@ -1200,34 +1200,34 @@
         <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>52</v>
+        <v>112</v>
       </c>
       <c r="T7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U7" t="n">
-        <v>997</v>
+        <v>1018</v>
       </c>
       <c r="V7" t="n">
-        <v>567</v>
+        <v>623</v>
       </c>
       <c r="W7" t="n">
-        <v>428</v>
+        <v>394</v>
       </c>
       <c r="X7" t="n">
-        <v>510</v>
+        <v>498</v>
       </c>
       <c r="Y7" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="Z7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AA7" t="n">
         <v>0</v>
       </c>
       <c r="AB7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC7" t="n">
         <v>0</v>
@@ -1236,16 +1236,16 @@
         <v>0</v>
       </c>
       <c r="AE7" t="n">
-        <v>52</v>
+        <v>112</v>
       </c>
       <c r="AF7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AG7" t="n">
-        <v>997</v>
+        <v>1018</v>
       </c>
       <c r="AH7" t="n">
-        <v>567</v>
+        <v>623</v>
       </c>
     </row>
     <row r="8">
@@ -1260,16 +1260,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>3453</v>
+        <v>3825</v>
       </c>
       <c r="D8" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="E8" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F8" t="n">
-        <v>277</v>
+        <v>311</v>
       </c>
       <c r="G8" t="n">
         <v>2</v>
@@ -1281,25 +1281,25 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>3480</v>
+        <v>3858</v>
       </c>
       <c r="K8" t="n">
-        <v>2210</v>
+        <v>2105</v>
       </c>
       <c r="L8" t="n">
-        <v>2073</v>
+        <v>1928</v>
       </c>
       <c r="M8" t="n">
-        <v>158</v>
+        <v>223</v>
       </c>
       <c r="N8" t="n">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="O8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q8" t="n">
         <v>2</v>
@@ -1308,34 +1308,34 @@
         <v>2</v>
       </c>
       <c r="S8" t="n">
-        <v>62</v>
+        <v>261</v>
       </c>
       <c r="T8" t="n">
+        <v>9</v>
+      </c>
+      <c r="U8" t="n">
+        <v>4573</v>
+      </c>
+      <c r="V8" t="n">
+        <v>2432</v>
+      </c>
+      <c r="W8" t="n">
+        <v>2100</v>
+      </c>
+      <c r="X8" t="n">
+        <v>1928</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>229</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>36</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB8" t="n">
         <v>2</v>
-      </c>
-      <c r="U8" t="n">
-        <v>4540</v>
-      </c>
-      <c r="V8" t="n">
-        <v>2305</v>
-      </c>
-      <c r="W8" t="n">
-        <v>2210</v>
-      </c>
-      <c r="X8" t="n">
-        <v>2074</v>
-      </c>
-      <c r="Y8" t="n">
-        <v>155</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>27</v>
-      </c>
-      <c r="AA8" t="n">
-        <v>6</v>
-      </c>
-      <c r="AB8" t="n">
-        <v>0</v>
       </c>
       <c r="AC8" t="n">
         <v>2</v>
@@ -1344,16 +1344,16 @@
         <v>2</v>
       </c>
       <c r="AE8" t="n">
-        <v>61</v>
+        <v>261</v>
       </c>
       <c r="AF8" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="AG8" t="n">
-        <v>4539</v>
+        <v>4574</v>
       </c>
       <c r="AH8" t="n">
-        <v>2302</v>
+        <v>2438</v>
       </c>
     </row>
     <row r="9">
@@ -1368,100 +1368,100 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>4500</v>
+        <v>5117</v>
       </c>
       <c r="D9" t="n">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="E9" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F9" t="n">
-        <v>211</v>
+        <v>242</v>
       </c>
       <c r="G9" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H9" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>4602</v>
+        <v>5227</v>
       </c>
       <c r="K9" t="n">
-        <v>3079</v>
+        <v>2889</v>
       </c>
       <c r="L9" t="n">
-        <v>2603</v>
+        <v>2279</v>
       </c>
       <c r="M9" t="n">
-        <v>42</v>
+        <v>139</v>
       </c>
       <c r="N9" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="O9" t="n">
-        <v>105</v>
+        <v>154</v>
       </c>
       <c r="P9" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="Q9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R9" t="n">
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>17</v>
+        <v>458</v>
       </c>
       <c r="T9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U9" t="n">
-        <v>5884</v>
+        <v>5969</v>
       </c>
       <c r="V9" t="n">
-        <v>2772</v>
+        <v>3042</v>
       </c>
       <c r="W9" t="n">
-        <v>3079</v>
+        <v>2890</v>
       </c>
       <c r="X9" t="n">
-        <v>2603</v>
+        <v>2279</v>
       </c>
       <c r="Y9" t="n">
-        <v>42</v>
+        <v>137</v>
       </c>
       <c r="Z9" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="AA9" t="n">
-        <v>105</v>
+        <v>153</v>
       </c>
       <c r="AB9" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="AC9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AD9" t="n">
         <v>0</v>
       </c>
       <c r="AE9" t="n">
-        <v>17</v>
+        <v>458</v>
       </c>
       <c r="AF9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG9" t="n">
-        <v>5884</v>
+        <v>5969</v>
       </c>
       <c r="AH9" t="n">
-        <v>2772</v>
+        <v>3040</v>
       </c>
     </row>
     <row r="10">
@@ -1476,19 +1476,19 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>5563</v>
+        <v>6338</v>
       </c>
       <c r="D10" t="n">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="E10" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F10" t="n">
-        <v>347</v>
+        <v>392</v>
       </c>
       <c r="G10" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="H10" t="n">
         <v>25</v>
@@ -1497,22 +1497,22 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>5703</v>
+        <v>6492</v>
       </c>
       <c r="K10" t="n">
-        <v>3915</v>
+        <v>3660</v>
       </c>
       <c r="L10" t="n">
-        <v>3813</v>
+        <v>3861</v>
       </c>
       <c r="M10" t="n">
-        <v>51</v>
+        <v>90</v>
       </c>
       <c r="N10" t="n">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="O10" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1524,31 +1524,31 @@
         <v>1</v>
       </c>
       <c r="S10" t="n">
-        <v>25</v>
+        <v>228</v>
       </c>
       <c r="T10" t="n">
         <v>3</v>
       </c>
       <c r="U10" t="n">
-        <v>7944</v>
+        <v>8009</v>
       </c>
       <c r="V10" t="n">
-        <v>3900</v>
+        <v>4199</v>
       </c>
       <c r="W10" t="n">
-        <v>3918</v>
+        <v>3661</v>
       </c>
       <c r="X10" t="n">
-        <v>3813</v>
+        <v>3854</v>
       </c>
       <c r="Y10" t="n">
-        <v>50</v>
+        <v>98</v>
       </c>
       <c r="Z10" t="n">
-        <v>126</v>
+        <v>150</v>
       </c>
       <c r="AA10" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="AB10" t="n">
         <v>0</v>
@@ -1560,16 +1560,16 @@
         <v>1</v>
       </c>
       <c r="AE10" t="n">
-        <v>25</v>
+        <v>227</v>
       </c>
       <c r="AF10" t="n">
         <v>3</v>
       </c>
       <c r="AG10" t="n">
-        <v>7944</v>
+        <v>8009</v>
       </c>
       <c r="AH10" t="n">
-        <v>3900</v>
+        <v>4198</v>
       </c>
     </row>
     <row r="11">
@@ -1584,16 +1584,16 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>4415</v>
+        <v>4960</v>
       </c>
       <c r="D11" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E11" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F11" t="n">
-        <v>299</v>
+        <v>345</v>
       </c>
       <c r="G11" t="n">
         <v>5</v>
@@ -1605,25 +1605,25 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>4452</v>
+        <v>4999</v>
       </c>
       <c r="K11" t="n">
-        <v>2373</v>
+        <v>2154</v>
       </c>
       <c r="L11" t="n">
-        <v>2316</v>
+        <v>2397</v>
       </c>
       <c r="M11" t="n">
-        <v>86</v>
+        <v>58</v>
       </c>
       <c r="N11" t="n">
-        <v>155</v>
+        <v>128</v>
       </c>
       <c r="O11" t="n">
-        <v>68</v>
+        <v>46</v>
       </c>
       <c r="P11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q11" t="n">
         <v>3</v>
@@ -1632,34 +1632,34 @@
         <v>0</v>
       </c>
       <c r="S11" t="n">
-        <v>116</v>
+        <v>371</v>
       </c>
       <c r="T11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U11" t="n">
-        <v>5119</v>
+        <v>5162</v>
       </c>
       <c r="V11" t="n">
-        <v>2591</v>
+        <v>2880</v>
       </c>
       <c r="W11" t="n">
-        <v>2373</v>
+        <v>2159</v>
       </c>
       <c r="X11" t="n">
-        <v>2314</v>
+        <v>2397</v>
       </c>
       <c r="Y11" t="n">
-        <v>88</v>
+        <v>52</v>
       </c>
       <c r="Z11" t="n">
-        <v>155</v>
+        <v>129</v>
       </c>
       <c r="AA11" t="n">
-        <v>68</v>
+        <v>46</v>
       </c>
       <c r="AB11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC11" t="n">
         <v>3</v>
@@ -1668,16 +1668,16 @@
         <v>0</v>
       </c>
       <c r="AE11" t="n">
-        <v>116</v>
+        <v>371</v>
       </c>
       <c r="AF11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AG11" t="n">
-        <v>5119</v>
+        <v>5162</v>
       </c>
       <c r="AH11" t="n">
-        <v>2591</v>
+        <v>2874</v>
       </c>
     </row>
     <row r="12">
@@ -1692,100 +1692,100 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1820</v>
+        <v>2246</v>
       </c>
       <c r="D12" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F12" t="n">
-        <v>102</v>
+        <v>130</v>
       </c>
       <c r="G12" t="n">
         <v>3</v>
       </c>
       <c r="H12" t="n">
+        <v>6</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>2279</v>
+      </c>
+      <c r="K12" t="n">
+        <v>1148</v>
+      </c>
+      <c r="L12" t="n">
+        <v>800</v>
+      </c>
+      <c r="M12" t="n">
+        <v>127</v>
+      </c>
+      <c r="N12" t="n">
+        <v>32</v>
+      </c>
+      <c r="O12" t="n">
+        <v>39</v>
+      </c>
+      <c r="P12" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q12" t="n">
         <v>3</v>
       </c>
-      <c r="I12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" t="n">
-        <v>1852</v>
-      </c>
-      <c r="K12" t="n">
-        <v>1273</v>
-      </c>
-      <c r="L12" t="n">
-        <v>899</v>
-      </c>
-      <c r="M12" t="n">
-        <v>88</v>
-      </c>
-      <c r="N12" t="n">
-        <v>30</v>
-      </c>
-      <c r="O12" t="n">
-        <v>22</v>
-      </c>
-      <c r="P12" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>2</v>
-      </c>
       <c r="R12" t="n">
         <v>0</v>
       </c>
       <c r="S12" t="n">
-        <v>63</v>
+        <v>229</v>
       </c>
       <c r="T12" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="U12" t="n">
-        <v>2383</v>
+        <v>2396</v>
       </c>
       <c r="V12" t="n">
-        <v>1080</v>
+        <v>1216</v>
       </c>
       <c r="W12" t="n">
-        <v>1274</v>
+        <v>1150</v>
       </c>
       <c r="X12" t="n">
-        <v>901</v>
+        <v>800</v>
       </c>
       <c r="Y12" t="n">
-        <v>87</v>
+        <v>127</v>
       </c>
       <c r="Z12" t="n">
         <v>30</v>
       </c>
       <c r="AA12" t="n">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="AB12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AD12" t="n">
         <v>0</v>
       </c>
       <c r="AE12" t="n">
-        <v>61</v>
+        <v>229</v>
       </c>
       <c r="AF12" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="AG12" t="n">
-        <v>2383</v>
+        <v>2396</v>
       </c>
       <c r="AH12" t="n">
-        <v>1079</v>
+        <v>1216</v>
       </c>
     </row>
     <row r="13">
@@ -1800,19 +1800,19 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>8373</v>
+        <v>9658</v>
       </c>
       <c r="D13" t="n">
-        <v>108</v>
+        <v>121</v>
       </c>
       <c r="E13" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F13" t="n">
-        <v>599</v>
+        <v>691</v>
       </c>
       <c r="G13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H13" t="n">
         <v>7</v>
@@ -1821,79 +1821,79 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>8481</v>
+        <v>9779</v>
       </c>
       <c r="K13" t="n">
-        <v>3667</v>
+        <v>3161</v>
       </c>
       <c r="L13" t="n">
-        <v>5078</v>
+        <v>5121</v>
       </c>
       <c r="M13" t="n">
-        <v>74</v>
+        <v>180</v>
       </c>
       <c r="N13" t="n">
-        <v>122</v>
+        <v>162</v>
       </c>
       <c r="O13" t="n">
-        <v>113</v>
+        <v>96</v>
       </c>
       <c r="P13" t="n">
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="R13" t="n">
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>185</v>
+        <v>710</v>
       </c>
       <c r="T13" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="U13" t="n">
-        <v>9254</v>
+        <v>9452</v>
       </c>
       <c r="V13" t="n">
-        <v>5465</v>
+        <v>6129</v>
       </c>
       <c r="W13" t="n">
-        <v>3402</v>
+        <v>2895</v>
       </c>
       <c r="X13" t="n">
-        <v>5075</v>
+        <v>5121</v>
       </c>
       <c r="Y13" t="n">
-        <v>69</v>
+        <v>179</v>
       </c>
       <c r="Z13" t="n">
-        <v>121</v>
+        <v>161</v>
       </c>
       <c r="AA13" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="AB13" t="n">
         <v>0</v>
       </c>
       <c r="AC13" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AD13" t="n">
         <v>0</v>
       </c>
       <c r="AE13" t="n">
-        <v>185</v>
+        <v>710</v>
       </c>
       <c r="AF13" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="AG13" t="n">
-        <v>8899</v>
+        <v>9097</v>
       </c>
       <c r="AH13" t="n">
-        <v>5376</v>
+        <v>6041</v>
       </c>
     </row>
     <row r="14">
@@ -1908,16 +1908,16 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1411</v>
+        <v>1630</v>
       </c>
       <c r="D14" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="E14" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F14" t="n">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G14" t="n">
         <v>1</v>
@@ -1929,22 +1929,22 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>1429</v>
+        <v>1653</v>
       </c>
       <c r="K14" t="n">
-        <v>361</v>
+        <v>319</v>
       </c>
       <c r="L14" t="n">
-        <v>713</v>
+        <v>664</v>
       </c>
       <c r="M14" t="n">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="N14" t="n">
         <v>0</v>
       </c>
       <c r="O14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P14" t="n">
         <v>0</v>
@@ -1956,31 +1956,31 @@
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>37</v>
+        <v>154</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
       </c>
       <c r="U14" t="n">
-        <v>1140</v>
+        <v>1152</v>
       </c>
       <c r="V14" t="n">
-        <v>779</v>
+        <v>833</v>
       </c>
       <c r="W14" t="n">
-        <v>361</v>
+        <v>319</v>
       </c>
       <c r="X14" t="n">
-        <v>713</v>
+        <v>664</v>
       </c>
       <c r="Y14" t="n">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="Z14" t="n">
         <v>0</v>
       </c>
       <c r="AA14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AB14" t="n">
         <v>0</v>
@@ -1992,16 +1992,16 @@
         <v>0</v>
       </c>
       <c r="AE14" t="n">
-        <v>37</v>
+        <v>154</v>
       </c>
       <c r="AF14" t="n">
         <v>0</v>
       </c>
       <c r="AG14" t="n">
-        <v>1140</v>
+        <v>1152</v>
       </c>
       <c r="AH14" t="n">
-        <v>779</v>
+        <v>833</v>
       </c>
     </row>
     <row r="15">
@@ -2016,7 +2016,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>494</v>
+        <v>512</v>
       </c>
       <c r="D15" t="n">
         <v>4</v>
@@ -2025,7 +2025,7 @@
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G15" t="n">
         <v>3</v>
@@ -2037,19 +2037,19 @@
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>498</v>
+        <v>516</v>
       </c>
       <c r="K15" t="n">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="L15" t="n">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="M15" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="N15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O15" t="n">
         <v>2</v>
@@ -2070,22 +2070,22 @@
         <v>0</v>
       </c>
       <c r="U15" t="n">
-        <v>601</v>
+        <v>622</v>
       </c>
       <c r="V15" t="n">
-        <v>366</v>
+        <v>390</v>
       </c>
       <c r="W15" t="n">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="X15" t="n">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="Y15" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="Z15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AA15" t="n">
         <v>2</v>
@@ -2106,10 +2106,10 @@
         <v>0</v>
       </c>
       <c r="AG15" t="n">
-        <v>601</v>
+        <v>622</v>
       </c>
       <c r="AH15" t="n">
-        <v>366</v>
+        <v>390</v>
       </c>
     </row>
     <row r="16">
@@ -2124,16 +2124,16 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2199</v>
+        <v>2561</v>
       </c>
       <c r="D16" t="n">
         <v>26</v>
       </c>
       <c r="E16" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F16" t="n">
-        <v>201</v>
+        <v>234</v>
       </c>
       <c r="G16" t="n">
         <v>3</v>
@@ -2145,79 +2145,79 @@
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>2225</v>
+        <v>2587</v>
       </c>
       <c r="K16" t="n">
-        <v>1347</v>
+        <v>1236</v>
       </c>
       <c r="L16" t="n">
-        <v>1255</v>
+        <v>1149</v>
       </c>
       <c r="M16" t="n">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="N16" t="n">
+        <v>4</v>
+      </c>
+      <c r="O16" t="n">
+        <v>1</v>
+      </c>
+      <c r="P16" t="n">
         <v>6</v>
       </c>
-      <c r="O16" t="n">
-        <v>1</v>
-      </c>
-      <c r="P16" t="n">
-        <v>0</v>
-      </c>
       <c r="Q16" t="n">
+        <v>7</v>
+      </c>
+      <c r="R16" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" t="n">
+        <v>355</v>
+      </c>
+      <c r="T16" t="n">
+        <v>3</v>
+      </c>
+      <c r="U16" t="n">
+        <v>2781</v>
+      </c>
+      <c r="V16" t="n">
+        <v>1541</v>
+      </c>
+      <c r="W16" t="n">
+        <v>1230</v>
+      </c>
+      <c r="X16" t="n">
+        <v>1127</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>4</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB16" t="n">
         <v>6</v>
       </c>
-      <c r="R16" t="n">
-        <v>0</v>
-      </c>
-      <c r="S16" t="n">
-        <v>104</v>
-      </c>
-      <c r="T16" t="n">
-        <v>1</v>
-      </c>
-      <c r="U16" t="n">
-        <v>2753</v>
-      </c>
-      <c r="V16" t="n">
-        <v>1400</v>
-      </c>
-      <c r="W16" t="n">
-        <v>1348</v>
-      </c>
-      <c r="X16" t="n">
-        <v>1255</v>
-      </c>
-      <c r="Y16" t="n">
-        <v>32</v>
-      </c>
-      <c r="Z16" t="n">
-        <v>6</v>
-      </c>
-      <c r="AA16" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB16" t="n">
-        <v>0</v>
-      </c>
       <c r="AC16" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AD16" t="n">
         <v>0</v>
       </c>
       <c r="AE16" t="n">
-        <v>104</v>
+        <v>404</v>
       </c>
       <c r="AF16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AG16" t="n">
-        <v>2753</v>
+        <v>2784</v>
       </c>
       <c r="AH16" t="n">
-        <v>1399</v>
+        <v>1550</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update hasil olahan data mikro SLS dari run_notebook
</commit_message>
<xml_diff>
--- a/research/fasih-dashboard-se2026/data_mikro_sls/Agregat_Kecamatan_ANGGOTA KELUARGA.xlsx
+++ b/research/fasih-dashboard-se2026/data_mikro_sls/Agregat_Kecamatan_ANGGOTA KELUARGA.xlsx
@@ -600,100 +600,100 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>5697</v>
+        <v>6881</v>
       </c>
       <c r="D2" t="n">
-        <v>99</v>
+        <v>112</v>
       </c>
       <c r="E2" t="n">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="F2" t="n">
-        <v>181</v>
+        <v>244</v>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H2" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>5796</v>
+        <v>6993</v>
       </c>
       <c r="K2" t="n">
-        <v>1169</v>
+        <v>643</v>
       </c>
       <c r="L2" t="n">
-        <v>2221</v>
+        <v>2752</v>
       </c>
       <c r="M2" t="n">
-        <v>72</v>
+        <v>40</v>
       </c>
       <c r="N2" t="n">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="O2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="P2" t="n">
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="R2" t="n">
         <v>3</v>
       </c>
       <c r="S2" t="n">
-        <v>589</v>
+        <v>730</v>
       </c>
       <c r="T2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="U2" t="n">
-        <v>4130</v>
+        <v>4258</v>
       </c>
       <c r="V2" t="n">
-        <v>2924</v>
+        <v>3560</v>
       </c>
       <c r="W2" t="n">
-        <v>1169</v>
+        <v>643</v>
       </c>
       <c r="X2" t="n">
-        <v>2221</v>
+        <v>2754</v>
       </c>
       <c r="Y2" t="n">
-        <v>72</v>
+        <v>40</v>
       </c>
       <c r="Z2" t="n">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="AA2" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="AB2" t="n">
         <v>0</v>
       </c>
       <c r="AC2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AD2" t="n">
         <v>3</v>
       </c>
       <c r="AE2" t="n">
-        <v>589</v>
+        <v>730</v>
       </c>
       <c r="AF2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="AG2" t="n">
-        <v>4130</v>
+        <v>4258</v>
       </c>
       <c r="AH2" t="n">
-        <v>2924</v>
+        <v>3560</v>
       </c>
     </row>
     <row r="3">
@@ -708,43 +708,43 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1239</v>
+        <v>1941</v>
       </c>
       <c r="D3" t="n">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="E3" t="n">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="F3" t="n">
-        <v>93</v>
+        <v>149</v>
       </c>
       <c r="G3" t="n">
         <v>1</v>
       </c>
       <c r="H3" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>1271</v>
+        <v>1984</v>
       </c>
       <c r="K3" t="n">
-        <v>410</v>
+        <v>184</v>
       </c>
       <c r="L3" t="n">
-        <v>507</v>
+        <v>857</v>
       </c>
       <c r="M3" t="n">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="N3" t="n">
-        <v>266</v>
+        <v>199</v>
       </c>
       <c r="O3" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="P3" t="n">
         <v>0</v>
@@ -756,31 +756,31 @@
         <v>1</v>
       </c>
       <c r="S3" t="n">
-        <v>202</v>
+        <v>212</v>
       </c>
       <c r="T3" t="n">
         <v>3</v>
       </c>
       <c r="U3" t="n">
-        <v>1420</v>
+        <v>1490</v>
       </c>
       <c r="V3" t="n">
-        <v>744</v>
+        <v>1107</v>
       </c>
       <c r="W3" t="n">
-        <v>410</v>
+        <v>184</v>
       </c>
       <c r="X3" t="n">
-        <v>507</v>
+        <v>857</v>
       </c>
       <c r="Y3" t="n">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="Z3" t="n">
-        <v>266</v>
+        <v>199</v>
       </c>
       <c r="AA3" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="AB3" t="n">
         <v>0</v>
@@ -792,16 +792,16 @@
         <v>1</v>
       </c>
       <c r="AE3" t="n">
-        <v>202</v>
+        <v>212</v>
       </c>
       <c r="AF3" t="n">
         <v>3</v>
       </c>
       <c r="AG3" t="n">
-        <v>1420</v>
+        <v>1490</v>
       </c>
       <c r="AH3" t="n">
-        <v>744</v>
+        <v>1107</v>
       </c>
     </row>
     <row r="4">
@@ -816,43 +816,43 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>6426</v>
+        <v>7789</v>
       </c>
       <c r="D4" t="n">
-        <v>93</v>
+        <v>123</v>
       </c>
       <c r="E4" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="F4" t="n">
-        <v>711</v>
+        <v>824</v>
       </c>
       <c r="G4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>6519</v>
+        <v>7912</v>
       </c>
       <c r="K4" t="n">
-        <v>1605</v>
+        <v>957</v>
       </c>
       <c r="L4" t="n">
-        <v>3789</v>
+        <v>4368</v>
       </c>
       <c r="M4" t="n">
-        <v>104</v>
+        <v>399</v>
       </c>
       <c r="N4" t="n">
-        <v>86</v>
+        <v>100</v>
       </c>
       <c r="O4" t="n">
-        <v>113</v>
+        <v>73</v>
       </c>
       <c r="P4" t="n">
         <v>0</v>
@@ -864,31 +864,31 @@
         <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>543</v>
+        <v>588</v>
       </c>
       <c r="T4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U4" t="n">
-        <v>6241</v>
+        <v>6487</v>
       </c>
       <c r="V4" t="n">
-        <v>4550</v>
+        <v>5430</v>
       </c>
       <c r="W4" t="n">
-        <v>1605</v>
+        <v>959</v>
       </c>
       <c r="X4" t="n">
-        <v>3789</v>
+        <v>4368</v>
       </c>
       <c r="Y4" t="n">
-        <v>104</v>
+        <v>399</v>
       </c>
       <c r="Z4" t="n">
-        <v>85</v>
+        <v>98</v>
       </c>
       <c r="AA4" t="n">
-        <v>113</v>
+        <v>73</v>
       </c>
       <c r="AB4" t="n">
         <v>0</v>
@@ -900,16 +900,16 @@
         <v>0</v>
       </c>
       <c r="AE4" t="n">
-        <v>543</v>
+        <v>588</v>
       </c>
       <c r="AF4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG4" t="n">
-        <v>6240</v>
+        <v>6487</v>
       </c>
       <c r="AH4" t="n">
-        <v>4550</v>
+        <v>5430</v>
       </c>
     </row>
     <row r="5">
@@ -924,100 +924,100 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>3763</v>
+        <v>4650</v>
       </c>
       <c r="D5" t="n">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="E5" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F5" t="n">
-        <v>215</v>
+        <v>253</v>
       </c>
       <c r="G5" t="n">
         <v>2</v>
       </c>
       <c r="H5" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>3833</v>
+        <v>4729</v>
       </c>
       <c r="K5" t="n">
-        <v>805</v>
+        <v>382</v>
       </c>
       <c r="L5" t="n">
-        <v>1886</v>
+        <v>2276</v>
       </c>
       <c r="M5" t="n">
+        <v>121</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="n">
+        <v>9</v>
+      </c>
+      <c r="P5" t="n">
+        <v>22</v>
+      </c>
+      <c r="Q5" t="n">
         <v>4</v>
       </c>
-      <c r="N5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" t="n">
-        <v>13</v>
-      </c>
-      <c r="P5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>2</v>
-      </c>
       <c r="R5" t="n">
         <v>0</v>
       </c>
       <c r="S5" t="n">
-        <v>440</v>
+        <v>488</v>
       </c>
       <c r="T5" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="U5" t="n">
-        <v>3158</v>
+        <v>3306</v>
       </c>
       <c r="V5" t="n">
-        <v>2353</v>
+        <v>2924</v>
       </c>
       <c r="W5" t="n">
-        <v>806</v>
+        <v>383</v>
       </c>
       <c r="X5" t="n">
-        <v>1886</v>
+        <v>2276</v>
       </c>
       <c r="Y5" t="n">
-        <v>3</v>
+        <v>120</v>
       </c>
       <c r="Z5" t="n">
         <v>0</v>
       </c>
       <c r="AA5" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="AB5" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="AC5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AD5" t="n">
         <v>0</v>
       </c>
       <c r="AE5" t="n">
-        <v>440</v>
+        <v>488</v>
       </c>
       <c r="AF5" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="AG5" t="n">
-        <v>3158</v>
+        <v>3306</v>
       </c>
       <c r="AH5" t="n">
-        <v>2352</v>
+        <v>2923</v>
       </c>
     </row>
     <row r="6">
@@ -1032,16 +1032,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1171</v>
+        <v>1468</v>
       </c>
       <c r="D6" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F6" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="G6" t="n">
         <v>3</v>
@@ -1053,22 +1053,22 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>1196</v>
+        <v>1494</v>
       </c>
       <c r="K6" t="n">
-        <v>421</v>
+        <v>310</v>
       </c>
       <c r="L6" t="n">
-        <v>558</v>
+        <v>694</v>
       </c>
       <c r="M6" t="n">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="N6" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="O6" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="P6" t="n">
         <v>0</v>
@@ -1080,31 +1080,31 @@
         <v>0</v>
       </c>
       <c r="S6" t="n">
-        <v>93</v>
+        <v>113</v>
       </c>
       <c r="T6" t="n">
+        <v>7</v>
+      </c>
+      <c r="U6" t="n">
+        <v>1158</v>
+      </c>
+      <c r="V6" t="n">
+        <v>832</v>
+      </c>
+      <c r="W6" t="n">
+        <v>310</v>
+      </c>
+      <c r="X6" t="n">
+        <v>694</v>
+      </c>
+      <c r="Y6" t="n">
         <v>8</v>
       </c>
-      <c r="U6" t="n">
-        <v>1134</v>
-      </c>
-      <c r="V6" t="n">
-        <v>693</v>
-      </c>
-      <c r="W6" t="n">
-        <v>422</v>
-      </c>
-      <c r="X6" t="n">
-        <v>558</v>
-      </c>
-      <c r="Y6" t="n">
-        <v>31</v>
-      </c>
       <c r="Z6" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="AA6" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="AB6" t="n">
         <v>0</v>
@@ -1116,16 +1116,16 @@
         <v>0</v>
       </c>
       <c r="AE6" t="n">
-        <v>92</v>
+        <v>113</v>
       </c>
       <c r="AF6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AG6" t="n">
-        <v>1134</v>
+        <v>1158</v>
       </c>
       <c r="AH6" t="n">
-        <v>692</v>
+        <v>832</v>
       </c>
     </row>
     <row r="7">
@@ -1140,16 +1140,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1072</v>
+        <v>1400</v>
       </c>
       <c r="D7" t="n">
-        <v>50</v>
+        <v>69</v>
       </c>
       <c r="E7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F7" t="n">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -1161,79 +1161,79 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>1122</v>
+        <v>1469</v>
       </c>
       <c r="K7" t="n">
-        <v>384</v>
+        <v>280</v>
       </c>
       <c r="L7" t="n">
-        <v>504</v>
+        <v>644</v>
       </c>
       <c r="M7" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="N7" t="n">
         <v>1</v>
       </c>
       <c r="O7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" t="n">
+        <v>133</v>
+      </c>
+      <c r="T7" t="n">
+        <v>5</v>
+      </c>
+      <c r="U7" t="n">
+        <v>1065</v>
+      </c>
+      <c r="V7" t="n">
+        <v>784</v>
+      </c>
+      <c r="W7" t="n">
+        <v>280</v>
+      </c>
+      <c r="X7" t="n">
+        <v>644</v>
+      </c>
+      <c r="Y7" t="n">
         <v>1</v>
-      </c>
-      <c r="R7" t="n">
-        <v>0</v>
-      </c>
-      <c r="S7" t="n">
-        <v>112</v>
-      </c>
-      <c r="T7" t="n">
-        <v>4</v>
-      </c>
-      <c r="U7" t="n">
-        <v>1019</v>
-      </c>
-      <c r="V7" t="n">
-        <v>634</v>
-      </c>
-      <c r="W7" t="n">
-        <v>384</v>
-      </c>
-      <c r="X7" t="n">
-        <v>504</v>
-      </c>
-      <c r="Y7" t="n">
-        <v>10</v>
       </c>
       <c r="Z7" t="n">
         <v>1</v>
       </c>
       <c r="AA7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AB7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD7" t="n">
         <v>0</v>
       </c>
       <c r="AE7" t="n">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="AF7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG7" t="n">
-        <v>1019</v>
+        <v>1065</v>
       </c>
       <c r="AH7" t="n">
-        <v>634</v>
+        <v>784</v>
       </c>
     </row>
     <row r="8">
@@ -1248,100 +1248,100 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>3944</v>
+        <v>5097</v>
       </c>
       <c r="D8" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="E8" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F8" t="n">
-        <v>323</v>
+        <v>398</v>
       </c>
       <c r="G8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H8" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>3977</v>
+        <v>5139</v>
       </c>
       <c r="K8" t="n">
-        <v>2049</v>
+        <v>1630</v>
       </c>
       <c r="L8" t="n">
-        <v>1986</v>
+        <v>2443</v>
       </c>
       <c r="M8" t="n">
-        <v>223</v>
+        <v>289</v>
       </c>
       <c r="N8" t="n">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="O8" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="P8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="R8" t="n">
         <v>2</v>
       </c>
       <c r="S8" t="n">
-        <v>277</v>
+        <v>378</v>
       </c>
       <c r="T8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U8" t="n">
-        <v>4596</v>
+        <v>4810</v>
       </c>
       <c r="V8" t="n">
-        <v>2510</v>
+        <v>3153</v>
       </c>
       <c r="W8" t="n">
-        <v>2049</v>
+        <v>1630</v>
       </c>
       <c r="X8" t="n">
-        <v>1990</v>
+        <v>2443</v>
       </c>
       <c r="Y8" t="n">
-        <v>220</v>
+        <v>289</v>
       </c>
       <c r="Z8" t="n">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="AA8" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="AB8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC8" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AD8" t="n">
         <v>2</v>
       </c>
       <c r="AE8" t="n">
-        <v>277</v>
+        <v>378</v>
       </c>
       <c r="AF8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AG8" t="n">
-        <v>4596</v>
+        <v>4810</v>
       </c>
       <c r="AH8" t="n">
-        <v>2510</v>
+        <v>3153</v>
       </c>
     </row>
     <row r="9">
@@ -1356,100 +1356,100 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>5342</v>
+        <v>7808</v>
       </c>
       <c r="D9" t="n">
-        <v>116</v>
+        <v>169</v>
       </c>
       <c r="E9" t="n">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="F9" t="n">
-        <v>253</v>
+        <v>348</v>
       </c>
       <c r="G9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H9" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>5458</v>
+        <v>7977</v>
       </c>
       <c r="K9" t="n">
-        <v>2813</v>
+        <v>1980</v>
       </c>
       <c r="L9" t="n">
-        <v>2427</v>
+        <v>3260</v>
       </c>
       <c r="M9" t="n">
-        <v>95</v>
+        <v>296</v>
       </c>
       <c r="N9" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="O9" t="n">
-        <v>95</v>
+        <v>198</v>
       </c>
       <c r="P9" t="n">
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R9" t="n">
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>531</v>
+        <v>577</v>
       </c>
       <c r="T9" t="n">
         <v>0</v>
       </c>
       <c r="U9" t="n">
-        <v>5997</v>
+        <v>6348</v>
       </c>
       <c r="V9" t="n">
-        <v>3149</v>
+        <v>4331</v>
       </c>
       <c r="W9" t="n">
-        <v>2808</v>
+        <v>1980</v>
       </c>
       <c r="X9" t="n">
-        <v>2424</v>
+        <v>3260</v>
       </c>
       <c r="Y9" t="n">
-        <v>103</v>
+        <v>295</v>
       </c>
       <c r="Z9" t="n">
         <v>37</v>
       </c>
       <c r="AA9" t="n">
-        <v>93</v>
+        <v>198</v>
       </c>
       <c r="AB9" t="n">
         <v>0</v>
       </c>
       <c r="AC9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD9" t="n">
         <v>0</v>
       </c>
       <c r="AE9" t="n">
-        <v>531</v>
+        <v>577</v>
       </c>
       <c r="AF9" t="n">
         <v>0</v>
       </c>
       <c r="AG9" t="n">
-        <v>5997</v>
+        <v>6347</v>
       </c>
       <c r="AH9" t="n">
-        <v>3152</v>
+        <v>4330</v>
       </c>
     </row>
     <row r="10">
@@ -1464,100 +1464,100 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>6706</v>
+        <v>8596</v>
       </c>
       <c r="D10" t="n">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="E10" t="n">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="F10" t="n">
-        <v>409</v>
+        <v>535</v>
       </c>
       <c r="G10" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="H10" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>6862</v>
+        <v>8779</v>
       </c>
       <c r="K10" t="n">
-        <v>3560</v>
+        <v>2620</v>
       </c>
       <c r="L10" t="n">
-        <v>3868</v>
+        <v>5034</v>
       </c>
       <c r="M10" t="n">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="N10" t="n">
-        <v>136</v>
+        <v>178</v>
       </c>
       <c r="O10" t="n">
+        <v>15</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>5</v>
+      </c>
+      <c r="R10" t="n">
+        <v>2</v>
+      </c>
+      <c r="S10" t="n">
+        <v>542</v>
+      </c>
+      <c r="T10" t="n">
         <v>6</v>
       </c>
-      <c r="P10" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>4</v>
-      </c>
-      <c r="R10" t="n">
-        <v>1</v>
-      </c>
-      <c r="S10" t="n">
-        <v>456</v>
-      </c>
-      <c r="T10" t="n">
+      <c r="U10" t="n">
+        <v>8450</v>
+      </c>
+      <c r="V10" t="n">
+        <v>5652</v>
+      </c>
+      <c r="W10" t="n">
+        <v>2620</v>
+      </c>
+      <c r="X10" t="n">
+        <v>5034</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>48</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>176</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>15</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC10" t="n">
         <v>5</v>
       </c>
-      <c r="U10" t="n">
-        <v>8064</v>
-      </c>
-      <c r="V10" t="n">
-        <v>4368</v>
-      </c>
-      <c r="W10" t="n">
-        <v>3560</v>
-      </c>
-      <c r="X10" t="n">
-        <v>3868</v>
-      </c>
-      <c r="Y10" t="n">
-        <v>28</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>136</v>
-      </c>
-      <c r="AA10" t="n">
+      <c r="AD10" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>542</v>
+      </c>
+      <c r="AF10" t="n">
         <v>6</v>
       </c>
-      <c r="AB10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC10" t="n">
-        <v>4</v>
-      </c>
-      <c r="AD10" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE10" t="n">
-        <v>456</v>
-      </c>
-      <c r="AF10" t="n">
-        <v>5</v>
-      </c>
       <c r="AG10" t="n">
-        <v>8064</v>
+        <v>8448</v>
       </c>
       <c r="AH10" t="n">
-        <v>4368</v>
+        <v>5652</v>
       </c>
     </row>
     <row r="11">
@@ -1572,19 +1572,19 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>5154</v>
+        <v>6839</v>
       </c>
       <c r="D11" t="n">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="E11" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F11" t="n">
-        <v>356</v>
+        <v>462</v>
       </c>
       <c r="G11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H11" t="n">
         <v>4</v>
@@ -1593,79 +1593,79 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>5194</v>
+        <v>6892</v>
       </c>
       <c r="K11" t="n">
-        <v>2077</v>
+        <v>1416</v>
       </c>
       <c r="L11" t="n">
-        <v>2487</v>
+        <v>3241</v>
       </c>
       <c r="M11" t="n">
-        <v>73</v>
+        <v>37</v>
       </c>
       <c r="N11" t="n">
-        <v>117</v>
+        <v>148</v>
       </c>
       <c r="O11" t="n">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="P11" t="n">
         <v>0</v>
       </c>
       <c r="Q11" t="n">
+        <v>6</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" t="n">
+        <v>453</v>
+      </c>
+      <c r="T11" t="n">
         <v>5</v>
       </c>
-      <c r="R11" t="n">
-        <v>0</v>
-      </c>
-      <c r="S11" t="n">
-        <v>371</v>
-      </c>
-      <c r="T11" t="n">
-        <v>4</v>
-      </c>
       <c r="U11" t="n">
-        <v>5177</v>
+        <v>5361</v>
       </c>
       <c r="V11" t="n">
-        <v>2983</v>
+        <v>3797</v>
       </c>
       <c r="W11" t="n">
-        <v>2077</v>
+        <v>1418</v>
       </c>
       <c r="X11" t="n">
-        <v>2487</v>
+        <v>3241</v>
       </c>
       <c r="Y11" t="n">
-        <v>73</v>
+        <v>35</v>
       </c>
       <c r="Z11" t="n">
-        <v>117</v>
+        <v>148</v>
       </c>
       <c r="AA11" t="n">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="AB11" t="n">
         <v>0</v>
       </c>
       <c r="AC11" t="n">
+        <v>6</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>453</v>
+      </c>
+      <c r="AF11" t="n">
         <v>5</v>
       </c>
-      <c r="AD11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE11" t="n">
-        <v>371</v>
-      </c>
-      <c r="AF11" t="n">
-        <v>4</v>
-      </c>
       <c r="AG11" t="n">
-        <v>5177</v>
+        <v>5361</v>
       </c>
       <c r="AH11" t="n">
-        <v>2983</v>
+        <v>3795</v>
       </c>
     </row>
     <row r="12">
@@ -1680,100 +1680,100 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2344</v>
+        <v>3240</v>
       </c>
       <c r="D12" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="E12" t="n">
+        <v>11</v>
+      </c>
+      <c r="F12" t="n">
+        <v>179</v>
+      </c>
+      <c r="G12" t="n">
+        <v>4</v>
+      </c>
+      <c r="H12" t="n">
+        <v>10</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>3286</v>
+      </c>
+      <c r="K12" t="n">
+        <v>751</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1250</v>
+      </c>
+      <c r="M12" t="n">
+        <v>13</v>
+      </c>
+      <c r="N12" t="n">
+        <v>86</v>
+      </c>
+      <c r="O12" t="n">
+        <v>70</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="n">
         <v>7</v>
       </c>
-      <c r="F12" t="n">
-        <v>131</v>
-      </c>
-      <c r="G12" t="n">
-        <v>3</v>
-      </c>
-      <c r="H12" t="n">
-        <v>6</v>
-      </c>
-      <c r="I12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" t="n">
-        <v>2378</v>
-      </c>
-      <c r="K12" t="n">
-        <v>1115</v>
-      </c>
-      <c r="L12" t="n">
-        <v>844</v>
-      </c>
-      <c r="M12" t="n">
-        <v>145</v>
-      </c>
-      <c r="N12" t="n">
-        <v>25</v>
-      </c>
-      <c r="O12" t="n">
-        <v>28</v>
-      </c>
-      <c r="P12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>3</v>
-      </c>
       <c r="R12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S12" t="n">
-        <v>230</v>
+        <v>249</v>
       </c>
       <c r="T12" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="U12" t="n">
-        <v>2406</v>
+        <v>2445</v>
       </c>
       <c r="V12" t="n">
-        <v>1266</v>
+        <v>1608</v>
       </c>
       <c r="W12" t="n">
-        <v>1115</v>
+        <v>751</v>
       </c>
       <c r="X12" t="n">
-        <v>841</v>
+        <v>1248</v>
       </c>
       <c r="Y12" t="n">
-        <v>148</v>
+        <v>15</v>
       </c>
       <c r="Z12" t="n">
-        <v>25</v>
+        <v>86</v>
       </c>
       <c r="AA12" t="n">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="AB12" t="n">
         <v>0</v>
       </c>
       <c r="AC12" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="AD12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE12" t="n">
-        <v>230</v>
+        <v>249</v>
       </c>
       <c r="AF12" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="AG12" t="n">
-        <v>2406</v>
+        <v>2445</v>
       </c>
       <c r="AH12" t="n">
-        <v>1266</v>
+        <v>1608</v>
       </c>
     </row>
     <row r="13">
@@ -1788,100 +1788,100 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>10348</v>
+        <v>13904</v>
       </c>
       <c r="D13" t="n">
-        <v>136</v>
+        <v>178</v>
       </c>
       <c r="E13" t="n">
-        <v>57</v>
+        <v>83</v>
       </c>
       <c r="F13" t="n">
-        <v>753</v>
+        <v>1004</v>
       </c>
       <c r="G13" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H13" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>10484</v>
+        <v>14082</v>
       </c>
       <c r="K13" t="n">
-        <v>2948</v>
+        <v>1393</v>
       </c>
       <c r="L13" t="n">
-        <v>5564</v>
+        <v>7134</v>
       </c>
       <c r="M13" t="n">
-        <v>109</v>
+        <v>54</v>
       </c>
       <c r="N13" t="n">
-        <v>99</v>
+        <v>147</v>
       </c>
       <c r="O13" t="n">
-        <v>94</v>
+        <v>10</v>
       </c>
       <c r="P13" t="n">
         <v>1</v>
       </c>
       <c r="Q13" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="R13" t="n">
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>719</v>
+        <v>969</v>
       </c>
       <c r="T13" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="U13" t="n">
-        <v>9558</v>
+        <v>9735</v>
       </c>
       <c r="V13" t="n">
-        <v>6511</v>
+        <v>8195</v>
       </c>
       <c r="W13" t="n">
-        <v>2682</v>
+        <v>1394</v>
       </c>
       <c r="X13" t="n">
-        <v>5561</v>
+        <v>7134</v>
       </c>
       <c r="Y13" t="n">
-        <v>112</v>
+        <v>54</v>
       </c>
       <c r="Z13" t="n">
-        <v>97</v>
+        <v>146</v>
       </c>
       <c r="AA13" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="AB13" t="n">
         <v>1</v>
       </c>
       <c r="AC13" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="AD13" t="n">
         <v>0</v>
       </c>
       <c r="AE13" t="n">
-        <v>719</v>
+        <v>969</v>
       </c>
       <c r="AF13" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AG13" t="n">
-        <v>9203</v>
+        <v>9735</v>
       </c>
       <c r="AH13" t="n">
-        <v>6424</v>
+        <v>8195</v>
       </c>
     </row>
     <row r="14">
@@ -1896,16 +1896,16 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1778</v>
+        <v>2266</v>
       </c>
       <c r="D14" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E14" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="F14" t="n">
-        <v>84</v>
+        <v>113</v>
       </c>
       <c r="G14" t="n">
         <v>1</v>
@@ -1917,16 +1917,16 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>1802</v>
+        <v>2292</v>
       </c>
       <c r="K14" t="n">
-        <v>269</v>
+        <v>99</v>
       </c>
       <c r="L14" t="n">
-        <v>723</v>
+        <v>891</v>
       </c>
       <c r="M14" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="N14" t="n">
         <v>0</v>
@@ -1944,25 +1944,25 @@
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>154</v>
+        <v>175</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
       </c>
       <c r="U14" t="n">
-        <v>1155</v>
+        <v>1190</v>
       </c>
       <c r="V14" t="n">
-        <v>886</v>
+        <v>1091</v>
       </c>
       <c r="W14" t="n">
-        <v>269</v>
+        <v>99</v>
       </c>
       <c r="X14" t="n">
-        <v>723</v>
+        <v>891</v>
       </c>
       <c r="Y14" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="Z14" t="n">
         <v>0</v>
@@ -1980,16 +1980,16 @@
         <v>0</v>
       </c>
       <c r="AE14" t="n">
-        <v>154</v>
+        <v>175</v>
       </c>
       <c r="AF14" t="n">
         <v>0</v>
       </c>
       <c r="AG14" t="n">
-        <v>1155</v>
+        <v>1190</v>
       </c>
       <c r="AH14" t="n">
-        <v>886</v>
+        <v>1091</v>
       </c>
     </row>
     <row r="15">
@@ -2004,7 +2004,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>519</v>
+        <v>529</v>
       </c>
       <c r="D15" t="n">
         <v>4</v>
@@ -2013,7 +2013,7 @@
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="G15" t="n">
         <v>3</v>
@@ -2025,19 +2025,19 @@
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>523</v>
+        <v>533</v>
       </c>
       <c r="K15" t="n">
-        <v>223</v>
+        <v>213</v>
       </c>
       <c r="L15" t="n">
-        <v>370</v>
+        <v>375</v>
       </c>
       <c r="M15" t="n">
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="O15" t="n">
         <v>3</v>
@@ -2052,28 +2052,28 @@
         <v>0</v>
       </c>
       <c r="S15" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="T15" t="n">
         <v>1</v>
       </c>
       <c r="U15" t="n">
-        <v>622</v>
+        <v>626</v>
       </c>
       <c r="V15" t="n">
-        <v>394</v>
+        <v>404</v>
       </c>
       <c r="W15" t="n">
-        <v>223</v>
+        <v>213</v>
       </c>
       <c r="X15" t="n">
-        <v>370</v>
+        <v>375</v>
       </c>
       <c r="Y15" t="n">
         <v>0</v>
       </c>
       <c r="Z15" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="AA15" t="n">
         <v>3</v>
@@ -2088,16 +2088,16 @@
         <v>0</v>
       </c>
       <c r="AE15" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="AF15" t="n">
         <v>1</v>
       </c>
       <c r="AG15" t="n">
-        <v>622</v>
+        <v>626</v>
       </c>
       <c r="AH15" t="n">
-        <v>394</v>
+        <v>404</v>
       </c>
     </row>
     <row r="16">
@@ -2112,46 +2112,46 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2712</v>
+        <v>3560</v>
       </c>
       <c r="D16" t="n">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="E16" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F16" t="n">
-        <v>250</v>
+        <v>312</v>
       </c>
       <c r="G16" t="n">
+        <v>6</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="n">
+        <v>3598</v>
+      </c>
+      <c r="K16" t="n">
+        <v>815</v>
+      </c>
+      <c r="L16" t="n">
+        <v>1522</v>
+      </c>
+      <c r="M16" t="n">
+        <v>53</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="n">
         <v>4</v>
       </c>
-      <c r="H16" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" t="n">
-        <v>2741</v>
-      </c>
-      <c r="K16" t="n">
-        <v>1162</v>
-      </c>
-      <c r="L16" t="n">
-        <v>1195</v>
-      </c>
-      <c r="M16" t="n">
-        <v>15</v>
-      </c>
-      <c r="N16" t="n">
-        <v>3</v>
-      </c>
-      <c r="O16" t="n">
-        <v>12</v>
-      </c>
       <c r="P16" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="Q16" t="n">
         <v>8</v>
@@ -2160,34 +2160,34 @@
         <v>0</v>
       </c>
       <c r="S16" t="n">
-        <v>407</v>
+        <v>492</v>
       </c>
       <c r="T16" t="n">
         <v>3</v>
       </c>
       <c r="U16" t="n">
-        <v>2805</v>
+        <v>2921</v>
       </c>
       <c r="V16" t="n">
-        <v>1640</v>
+        <v>2106</v>
       </c>
       <c r="W16" t="n">
-        <v>1163</v>
+        <v>815</v>
       </c>
       <c r="X16" t="n">
-        <v>1195</v>
+        <v>1522</v>
       </c>
       <c r="Y16" t="n">
-        <v>13</v>
+        <v>53</v>
       </c>
       <c r="Z16" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AA16" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="AB16" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="AC16" t="n">
         <v>8</v>
@@ -2196,16 +2196,16 @@
         <v>0</v>
       </c>
       <c r="AE16" t="n">
-        <v>407</v>
+        <v>492</v>
       </c>
       <c r="AF16" t="n">
         <v>3</v>
       </c>
       <c r="AG16" t="n">
-        <v>2804</v>
+        <v>2921</v>
       </c>
       <c r="AH16" t="n">
-        <v>1638</v>
+        <v>2106</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update hasil analisa notebook pengecekan SLS & data mikro SLS
</commit_message>
<xml_diff>
--- a/research/fasih-dashboard-se2026/data_mikro_sls/Agregat_Kecamatan_ANGGOTA KELUARGA.xlsx
+++ b/research/fasih-dashboard-se2026/data_mikro_sls/Agregat_Kecamatan_ANGGOTA KELUARGA.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,172 +429,172 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Kode Kecamatan</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Nama Kecamatan</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Tinggal Bersama Keluarga</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Anggota Keluarga Baru</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Meninggal</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Pindah Dalam Negeri (DN)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Pindah Luar Negeri (LN)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Tidak Ditemukan</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Anggota Keluarga Khusus</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Total Anggota Keluarga ((3) + (4))</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Scraped_Pencacah_OPEN</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Scraped_Pencacah_APPROVED BY Pengawas</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Scraped_Pencacah_SUBMITTED BY Pencacah</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Scraped_Pencacah_DRAFT</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Scraped_Pencacah_REJECTED BY Pengawas</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Scraped_Pencacah_REJECTED BY Admin Kabupaten</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Scraped_Pencacah_REVOKED BY Pengawas</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Scraped_Pencacah_SUBMITTED RESPONDENT</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Scraped_Pencacah_COMPLETED BY Admin Kabupaten</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Scraped_Pencacah_EDITED BY Admin Kabupaten</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Scraped_Pencacah_Total_Prelist_Scraped</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Scraped_Pencacah_Realisasi_Scraped</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Scraped_Pengawas_OPEN</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Scraped_Pengawas_APPROVED BY Pengawas</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Scraped_Pengawas_SUBMITTED BY Pencacah</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Scraped_Pengawas_DRAFT</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Scraped_Pengawas_REJECTED BY Pengawas</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Scraped_Pengawas_REJECTED BY Admin Kabupaten</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Scraped_Pengawas_REVOKED BY Pengawas</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Scraped_Pengawas_SUBMITTED RESPONDENT</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Scraped_Pengawas_COMPLETED BY Admin Kabupaten</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Scraped_Pengawas_EDITED BY Admin Kabupaten</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Scraped_Pengawas_Total_Prelist_Scraped</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Scraped_Pengawas_Realisasi_Scraped</t>
         </is>

</xml_diff>

<commit_message>
Fix notebook mapping petugas dari dashboard_scraped_data_evening.csv
</commit_message>
<xml_diff>
--- a/research/fasih-dashboard-se2026/data_mikro_sls/Agregat_Kecamatan_ANGGOTA KELUARGA.xlsx
+++ b/research/fasih-dashboard-se2026/data_mikro_sls/Agregat_Kecamatan_ANGGOTA KELUARGA.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,172 +417,172 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Kode Kecamatan</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Nama Kecamatan</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Tinggal Bersama Keluarga</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Anggota Keluarga Baru</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Meninggal</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Pindah Dalam Negeri (DN)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Pindah Luar Negeri (LN)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Tidak Ditemukan</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Anggota Keluarga Khusus</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Total Anggota Keluarga ((3) + (4))</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Scraped_Pencacah_OPEN</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Scraped_Pencacah_APPROVED BY Pengawas</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Scraped_Pencacah_SUBMITTED BY Pencacah</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Scraped_Pencacah_DRAFT</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Scraped_Pencacah_REJECTED BY Pengawas</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Scraped_Pencacah_REJECTED BY Admin Kabupaten</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Scraped_Pencacah_REVOKED BY Pengawas</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Scraped_Pencacah_SUBMITTED RESPONDENT</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Scraped_Pencacah_COMPLETED BY Admin Kabupaten</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Scraped_Pencacah_EDITED BY Admin Kabupaten</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Scraped_Pencacah_Total_Prelist_Scraped</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Scraped_Pencacah_Realisasi_Scraped</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Scraped_Pengawas_OPEN</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Scraped_Pengawas_APPROVED BY Pengawas</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Scraped_Pengawas_SUBMITTED BY Pencacah</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Scraped_Pengawas_DRAFT</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>Scraped_Pengawas_REJECTED BY Pengawas</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>Scraped_Pengawas_REJECTED BY Admin Kabupaten</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>Scraped_Pengawas_REVOKED BY Pengawas</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>Scraped_Pengawas_SUBMITTED RESPONDENT</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>Scraped_Pengawas_COMPLETED BY Admin Kabupaten</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>Scraped_Pengawas_EDITED BY Admin Kabupaten</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>Scraped_Pengawas_Total_Prelist_Scraped</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>Scraped_Pengawas_Realisasi_Scraped</t>
         </is>

</xml_diff>